<commit_message>
Election system updates and print layout improvements
:wq#
</commit_message>
<xml_diff>
--- a/static/uploads/LIST.xlsx
+++ b/static/uploads/LIST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/75bcf1cf94a9ee92/Desktop/voting_web/static/uploads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\voting_web\static\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{DD801695-FCBC-45EC-8784-A9E8D85AD28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37F98858-2E25-49BA-926F-67691A03E582}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C55E7C-8A2A-4F80-BE02-9015A12969E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5115" yWindow="3015" windowWidth="15375" windowHeight="7785" xr2:uid="{73CE7595-C661-4929-A0F4-5BA63C47C7A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{73CE7595-C661-4929-A0F4-5BA63C47C7A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
   <si>
     <t>ACKAH SYLVESTER EBI</t>
   </si>
@@ -146,10 +146,25 @@
     <t xml:space="preserve">AWIDANI MOSES </t>
   </si>
   <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>AGRREY</t>
+  </si>
+  <si>
+    <t>PADMORE</t>
+  </si>
+  <si>
+    <t>OKUMDOM</t>
+  </si>
+  <si>
+    <t>TANO</t>
+  </si>
+  <si>
     <t>student_id</t>
   </si>
   <si>
-    <t>name</t>
+    <t>group_name</t>
   </si>
 </sst>
 </file>
@@ -521,299 +536,408 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E015DF-1F62-413C-9F15-71BBB38FEF18}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="B25" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="B27" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="B28" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="B29" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
         <v>34</v>
+      </c>
+      <c r="C36" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>